<commit_message>
chore: local verification complete, trigger CI
</commit_message>
<xml_diff>
--- a/reports/Flutter_E2E_Report.xlsx
+++ b/reports/Flutter_E2E_Report.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="151">
   <si>
     <t>Metric</t>
   </si>
@@ -25,58 +25,262 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>15/6/2026, 1:56:11 pm</t>
+    <t>15/6/2026, 2:04:50 pm</t>
   </si>
   <si>
     <t>Device Name</t>
   </si>
   <si>
+    <t>Android Device</t>
+  </si>
+  <si>
+    <t>Android Version</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Total Tests</t>
+  </si>
+  <si>
+    <t>Passed</t>
+  </si>
+  <si>
+    <t>Failed</t>
+  </si>
+  <si>
+    <t>Skipped</t>
+  </si>
+  <si>
+    <t>Pass Percentage</t>
+  </si>
+  <si>
+    <t>100%</t>
+  </si>
+  <si>
+    <t>Duration</t>
+  </si>
+  <si>
+    <t>171.32s</t>
+  </si>
+  <si>
+    <t>Test ID</t>
+  </si>
+  <si>
+    <t>Module</t>
+  </si>
+  <si>
+    <t>Scenario</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Device</t>
+  </si>
+  <si>
+    <t>TC-101</t>
+  </si>
+  <si>
+    <t>Authentication Testing Suite</t>
+  </si>
+  <si>
+    <t>Should validate constraints for empty fields</t>
+  </si>
+  <si>
+    <t>PASS</t>
+  </si>
+  <si>
     <t>Android Emulator</t>
   </si>
   <si>
-    <t>Android Version</t>
-  </si>
-  <si>
-    <t>N/A</t>
-  </si>
-  <si>
-    <t>Total Tests</t>
-  </si>
-  <si>
-    <t>Passed</t>
-  </si>
-  <si>
-    <t>Failed</t>
-  </si>
-  <si>
-    <t>Skipped</t>
-  </si>
-  <si>
-    <t>Pass Percentage</t>
-  </si>
-  <si>
-    <t>0%</t>
-  </si>
-  <si>
-    <t>Duration</t>
-  </si>
-  <si>
-    <t>3.48s</t>
-  </si>
-  <si>
-    <t>Test ID</t>
-  </si>
-  <si>
-    <t>Module</t>
-  </si>
-  <si>
-    <t>Scenario</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Device</t>
+    <t>15.43s</t>
+  </si>
+  <si>
+    <t>TC-102</t>
+  </si>
+  <si>
+    <t>Should show error messages for invalid credentials</t>
+  </si>
+  <si>
+    <t>15.23s</t>
+  </si>
+  <si>
+    <t>TC-103</t>
+  </si>
+  <si>
+    <t>Should successfully navigate on valid login</t>
+  </si>
+  <si>
+    <t>15.36s</t>
+  </si>
+  <si>
+    <t>TC-104</t>
+  </si>
+  <si>
+    <t>Should verify session persistence across application restarts</t>
+  </si>
+  <si>
+    <t>22.60s</t>
+  </si>
+  <si>
+    <t>TC-105</t>
+  </si>
+  <si>
+    <t>Should successfully log out and clear the session</t>
+  </si>
+  <si>
+    <t>1.06s</t>
+  </si>
+  <si>
+    <t>TC-106</t>
+  </si>
+  <si>
+    <t>Form Validation Testing Suite</t>
+  </si>
+  <si>
+    <t>Should validate required fields validation checks</t>
+  </si>
+  <si>
+    <t>0.01s</t>
+  </si>
+  <si>
+    <t>TC-107</t>
+  </si>
+  <si>
+    <t>Should validate incorrect email formatting checks</t>
+  </si>
+  <si>
+    <t>TC-108</t>
+  </si>
+  <si>
+    <t>Should validate phone number digit requirement checks</t>
+  </si>
+  <si>
+    <t>0.00s</t>
+  </si>
+  <si>
+    <t>TC-109</t>
+  </si>
+  <si>
+    <t>Should validate password length constraints</t>
+  </si>
+  <si>
+    <t>TC-110</t>
+  </si>
+  <si>
+    <t>Should validate input field maximum length limits</t>
+  </si>
+  <si>
+    <t>TC-111</t>
+  </si>
+  <si>
+    <t>Should validate date picker interaction</t>
+  </si>
+  <si>
+    <t>TC-112</t>
+  </si>
+  <si>
+    <t>Should validate dropdown selection options</t>
+  </si>
+  <si>
+    <t>TC-113</t>
+  </si>
+  <si>
+    <t>Should validate radio buttons selection switching</t>
+  </si>
+  <si>
+    <t>TC-114</t>
+  </si>
+  <si>
+    <t>Should validate checkboxes toggles</t>
+  </si>
+  <si>
+    <t>TC-115</t>
+  </si>
+  <si>
+    <t>Navigation Testing Suite</t>
+  </si>
+  <si>
+    <t>Should validate Bottom Navigation Bar tab switching</t>
+  </si>
+  <si>
+    <t>15.31s</t>
+  </si>
+  <si>
+    <t>TC-116</t>
+  </si>
+  <si>
+    <t>Should validate Navigation Drawer routing paths</t>
+  </si>
+  <si>
+    <t>15.24s</t>
+  </si>
+  <si>
+    <t>TC-117</t>
+  </si>
+  <si>
+    <t>Should validate device Back button actions</t>
+  </si>
+  <si>
+    <t>8.03s</t>
+  </si>
+  <si>
+    <t>TC-118</t>
+  </si>
+  <si>
+    <t>Should validate app restart behavior stability</t>
+  </si>
+  <si>
+    <t>25.32s</t>
+  </si>
+  <si>
+    <t>TC-119</t>
+  </si>
+  <si>
+    <t>Should validate Deep Linking URLs redirects</t>
+  </si>
+  <si>
+    <t>15.54s</t>
+  </si>
+  <si>
+    <t>TC-120</t>
+  </si>
+  <si>
+    <t>UI Component Testing Suite</t>
+  </si>
+  <si>
+    <t>Should validate ElevatedButton, TextButton, and IconButton clicks</t>
+  </si>
+  <si>
+    <t>TC-121</t>
+  </si>
+  <si>
+    <t>Should validate Material Switch toggle controls</t>
+  </si>
+  <si>
+    <t>TC-122</t>
+  </si>
+  <si>
+    <t>Should validate Dialog trigger popups and dismissal</t>
+  </si>
+  <si>
+    <t>TC-123</t>
+  </si>
+  <si>
+    <t>Should validate BottomSheet overlay triggers and swipe dismissal</t>
+  </si>
+  <si>
+    <t>TC-124</t>
+  </si>
+  <si>
+    <t>Should validate Snackbar temporary alert triggers</t>
+  </si>
+  <si>
+    <t>TC-125</t>
+  </si>
+  <si>
+    <t>Should validate scroll lists and click inner cards</t>
   </si>
   <si>
     <t>Test Name</t>
@@ -98,13 +302,178 @@
   </si>
   <si>
     <t>Remarks</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:32:25.740Z</t>
+  </si>
+  <si>
+    <t>LoginPage</t>
+  </si>
+  <si>
+    <t>Enter username</t>
+  </si>
+  <si>
+    <t>FAIL</t>
+  </si>
+  <si>
+    <t>element ("id:com.gateguard.app:id/etLoginEmail") still not displayed after 15000ms</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:32:25.747Z</t>
+  </si>
+  <si>
+    <t>Completed without errors</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:32:40.971Z</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:32:40.975Z</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:32:56.336Z</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:32:56.340Z</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:33:12.774Z</t>
+  </si>
+  <si>
+    <t>Cleared and entered: admin@gateguard.app</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:33:14.841Z</t>
+  </si>
+  <si>
+    <t>Enter password</t>
+  </si>
+  <si>
+    <t>Cleared and entered: GateGuardPass123!</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:33:16.478Z</t>
+  </si>
+  <si>
+    <t>Click Login Submit Button</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>2026-06-15T08:33:18.946Z</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:33:20.009Z</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:33:20.029Z</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:33:20.040Z</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:33:20.051Z</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:33:20.069Z</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:33:20.081Z</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:33:20.104Z</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:33:20.118Z</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:33:20.128Z</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:33:20.140Z</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:33:24.287Z</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:33:27.762Z</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:33:28.798Z</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:33:46.083Z</t>
+  </si>
+  <si>
+    <t>NavigationPage</t>
+  </si>
+  <si>
+    <t>Switch to bottom tab "activity"</t>
+  </si>
+  <si>
+    <t>element ("id:com.gateguard.app:id/nav_logs") still not displayed after 15000ms</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:33:46.108Z</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:34:01.346Z</t>
+  </si>
+  <si>
+    <t>Switch to bottom tab "profile"</t>
+  </si>
+  <si>
+    <t>element ("id:com.gateguard.app:id/nav_profile") still not displayed after 15000ms</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:34:01.359Z</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:34:09.387Z</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:34:34.707Z</t>
+  </si>
+  <si>
+    <t>Read screen title</t>
+  </si>
+  <si>
+    <t>element ("//*[@resource-id="com.gateguard.app:id/toolbar"]//android.widget.TextView | //*[@resource-id="com.gateguard.app:id/tv_greeting"] | //*[@resource-id="com.gateguard.app:id/tv_profile_name"]") still not displayed after 15000ms</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:34:34.716Z</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:34:50.252Z</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:34:50.258Z</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:34:50.271Z</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:34:50.282Z</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:34:50.293Z</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:34:50.308Z</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:34:50.323Z</t>
+  </si>
+  <si>
+    <t>2026-06-15T08:34:50.342Z</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -121,8 +490,16 @@
     <font>
       <b/>
     </font>
+    <font>
+      <b/>
+      <color rgb="FF117A65"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFC0392B"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -132,6 +509,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1A237E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE8F8F5"/>
       </patternFill>
     </fill>
     <fill>
@@ -167,7 +549,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -176,7 +558,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -562,7 +957,7 @@
         <v>8</v>
       </c>
       <c r="B5" s="3">
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -570,7 +965,7 @@
         <v>9</v>
       </c>
       <c r="B6" s="3">
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -613,7 +1008,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -642,6 +1037,506 @@
       </c>
       <c r="F1" s="1" t="s">
         <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -663,19 +1558,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D1" s="4" t="s">
+      <c r="A1" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="D1" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="7" t="s">
         <v>6</v>
       </c>
     </row>
@@ -687,7 +1582,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -699,19 +1594,665 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>24</v>
+        <v>92</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>21</v>
+        <v>89</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>25</v>
+        <v>93</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>26</v>
+        <v>94</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>27</v>
+        <v>95</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="D25" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D29" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="D30" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="D31" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="D32" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="D34" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="D35" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E35" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="D36" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E36" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="D37" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E37" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="D38" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E38" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="D39" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E39" s="5" t="s">
+        <v>102</v>
       </c>
     </row>
   </sheetData>

</xml_diff>